<commit_message>
BC Answer keys updated
</commit_message>
<xml_diff>
--- a/Data/BC/BC_Quizzes.xlsx
+++ b/Data/BC/BC_Quizzes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\mba\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\mba\Data\BC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E8CD4ED-0054-4208-BFB0-AE04B28F8805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1980238-702F-4BCA-BD97-8B0DE97DE7D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="4" activeTab="11" xr2:uid="{A23BC9EF-D06A-4304-B965-EA8D9AB19B1B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A23BC9EF-D06A-4304-B965-EA8D9AB19B1B}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1491" uniqueCount="1063">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="1069">
   <si>
     <t>The exchange of information between people outside a company to achieve a fundamental goal.</t>
   </si>
@@ -3236,6 +3236,24 @@
   </si>
   <si>
     <t>Which of the following is an important aspect of the job interview process?</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -3359,7 +3377,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -3373,6 +3391,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3708,14 +3729,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE8C4031-046B-4647-A379-B4536C1E8D1D}">
   <sheetPr codeName="Sheet14"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="81.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -3734,8 +3755,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -3754,8 +3778,11 @@
       <c r="F2" s="4" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -3774,8 +3801,11 @@
       <c r="F3" s="7" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -3794,8 +3824,11 @@
       <c r="F4" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -3814,8 +3847,11 @@
       <c r="F5" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -3834,8 +3870,11 @@
       <c r="F6" s="7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -3854,8 +3893,11 @@
       <c r="F7" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -3874,8 +3916,11 @@
       <c r="F8" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -3894,8 +3939,11 @@
       <c r="F9" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -3914,8 +3962,11 @@
       <c r="F10" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -3934,8 +3985,11 @@
       <c r="F11" s="7" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -3954,8 +4008,11 @@
       <c r="F12" s="4" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -3974,8 +4031,11 @@
       <c r="F13" s="7" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -3994,8 +4054,11 @@
       <c r="F14" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -4014,8 +4077,11 @@
       <c r="F15" s="7" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -4034,8 +4100,11 @@
       <c r="F16" s="4" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -4054,8 +4123,11 @@
       <c r="F17" s="7" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -4074,8 +4146,11 @@
       <c r="F18" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -4094,8 +4169,11 @@
       <c r="F19" s="7" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -4114,8 +4192,11 @@
       <c r="F20" s="4" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -4133,6 +4214,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>42</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1064</v>
       </c>
     </row>
   </sheetData>
@@ -4143,7 +4227,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{501AAE18-B6BE-4AA9-A58C-D084CA656346}">
   <sheetPr codeName="Sheet17"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -4153,7 +4237,7 @@
     <col min="6" max="6" width="81.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -4172,8 +4256,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -4192,8 +4279,11 @@
       <c r="F2" s="4" t="s">
         <v>828</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -4212,8 +4302,11 @@
       <c r="F3" s="7" t="s">
         <v>838</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -4232,8 +4325,11 @@
       <c r="F4" s="7" t="s">
         <v>828</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -4252,8 +4348,11 @@
       <c r="F5" s="4" t="s">
         <v>824</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -4272,8 +4371,11 @@
       <c r="F6" s="7" t="s">
         <v>820</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -4292,8 +4394,11 @@
       <c r="F7" s="4" t="s">
         <v>815</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -4312,8 +4417,11 @@
       <c r="F8" s="7" t="s">
         <v>810</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -4332,8 +4440,11 @@
       <c r="F9" s="4" t="s">
         <v>805</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -4352,8 +4463,11 @@
       <c r="F10" s="1" t="s">
         <v>800</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -4372,8 +4486,11 @@
       <c r="F11" s="7" t="s">
         <v>881</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -4392,8 +4509,11 @@
       <c r="F12" s="4" t="s">
         <v>877</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -4412,8 +4532,11 @@
       <c r="F13" s="7" t="s">
         <v>872</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -4432,8 +4555,11 @@
       <c r="F14" s="4" t="s">
         <v>867</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -4452,8 +4578,11 @@
       <c r="F15" s="7" t="s">
         <v>862</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -4472,8 +4601,11 @@
       <c r="F16" s="4" t="s">
         <v>829</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -4492,8 +4624,11 @@
       <c r="F17" s="7" t="s">
         <v>855</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -4512,8 +4647,11 @@
       <c r="F18" s="4" t="s">
         <v>850</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -4532,8 +4670,11 @@
       <c r="F19" s="7" t="s">
         <v>847</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -4552,8 +4693,11 @@
       <c r="F20" s="4" t="s">
         <v>843</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -4571,6 +4715,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>833</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1067</v>
       </c>
     </row>
   </sheetData>
@@ -4581,7 +4728,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{621D6439-8B87-4595-89DD-63114212A034}">
   <sheetPr codeName="Sheet16"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -4592,7 +4739,7 @@
     <col min="6" max="6" width="65.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -4611,8 +4758,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -4631,8 +4781,11 @@
       <c r="F2" s="4" t="s">
         <v>890</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -4651,8 +4804,11 @@
       <c r="F3" s="7" t="s">
         <v>924</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -4671,8 +4827,11 @@
       <c r="F4" s="7" t="s">
         <v>888</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -4691,8 +4850,11 @@
       <c r="F5" s="4" t="s">
         <v>911</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -4711,8 +4873,11 @@
       <c r="F6" s="7" t="s">
         <v>906</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -4731,8 +4896,11 @@
       <c r="F7" s="4" t="s">
         <v>901</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -4751,8 +4919,11 @@
       <c r="F8" s="7" t="s">
         <v>897</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -4771,8 +4942,11 @@
       <c r="F9" s="4" t="s">
         <v>892</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -4791,8 +4965,11 @@
       <c r="F10" s="1" t="s">
         <v>887</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -4811,8 +4988,11 @@
       <c r="F11" s="7" t="s">
         <v>960</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -4831,8 +5011,11 @@
       <c r="F12" s="4" t="s">
         <v>967</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -4851,8 +5034,11 @@
       <c r="F13" s="7" t="s">
         <v>962</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -4871,8 +5057,11 @@
       <c r="F14" s="4" t="s">
         <v>887</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -4891,8 +5080,11 @@
       <c r="F15" s="7" t="s">
         <v>953</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -4911,8 +5103,11 @@
       <c r="F16" s="4" t="s">
         <v>948</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -4931,8 +5126,11 @@
       <c r="F17" s="7" t="s">
         <v>943</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -4951,8 +5149,11 @@
       <c r="F18" s="4" t="s">
         <v>939</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -4971,8 +5172,11 @@
       <c r="F19" s="7" t="s">
         <v>934</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -4991,8 +5195,11 @@
       <c r="F20" s="4" t="s">
         <v>929</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -5010,6 +5217,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>919</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1065</v>
       </c>
     </row>
   </sheetData>
@@ -5020,7 +5230,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD8264CE-5C5F-48EF-87DC-8BEAFE9054AF}">
   <sheetPr codeName="Sheet15"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -5031,7 +5241,7 @@
     <col min="6" max="6" width="67.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -5050,8 +5260,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -5070,8 +5283,11 @@
       <c r="F2" s="4" t="s">
         <v>1059</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -5090,8 +5306,11 @@
       <c r="F3" s="7" t="s">
         <v>1012</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -5110,8 +5329,11 @@
       <c r="F4" s="7" t="s">
         <v>1002</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -5130,8 +5352,11 @@
       <c r="F5" s="4" t="s">
         <v>998</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -5150,8 +5375,11 @@
       <c r="F6" s="7" t="s">
         <v>993</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -5170,8 +5398,11 @@
       <c r="F7" s="4" t="s">
         <v>988</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -5190,8 +5421,11 @@
       <c r="F8" s="7" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -5210,8 +5444,11 @@
       <c r="F9" s="4" t="s">
         <v>978</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -5230,8 +5467,11 @@
       <c r="F10" s="1" t="s">
         <v>973</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -5250,8 +5490,11 @@
       <c r="F11" s="7" t="s">
         <v>1054</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -5270,8 +5513,11 @@
       <c r="F12" s="4" t="s">
         <v>1045</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -5290,8 +5536,11 @@
       <c r="F13" s="7" t="s">
         <v>1045</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -5310,8 +5559,11 @@
       <c r="F14" s="4" t="s">
         <v>976</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -5330,8 +5582,11 @@
       <c r="F15" s="7" t="s">
         <v>1039</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -5350,8 +5605,11 @@
       <c r="F16" s="4" t="s">
         <v>1034</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -5370,8 +5628,11 @@
       <c r="F17" s="7" t="s">
         <v>1030</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -5390,8 +5651,11 @@
       <c r="F18" s="4" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -5410,8 +5674,11 @@
       <c r="F19" s="7" t="s">
         <v>1022</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -5430,8 +5697,11 @@
       <c r="F20" s="4" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -5449,6 +5719,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>1007</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1065</v>
       </c>
     </row>
   </sheetData>
@@ -5459,7 +5732,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{770A45F1-03D0-4C60-BA06-4D56BB255CF6}">
   <sheetPr codeName="Sheet13"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -5470,7 +5743,7 @@
     <col min="6" max="6" width="49.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -5489,8 +5762,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -5509,8 +5785,11 @@
       <c r="F2" s="4" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -5529,8 +5808,11 @@
       <c r="F3" s="7" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -5549,8 +5831,11 @@
       <c r="F4" s="7" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -5569,8 +5854,11 @@
       <c r="F5" s="4" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -5589,8 +5877,11 @@
       <c r="F6" s="7" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -5609,8 +5900,11 @@
       <c r="F7" s="4" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -5629,8 +5923,11 @@
       <c r="F8" s="7" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -5649,8 +5946,11 @@
       <c r="F9" s="4" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -5669,8 +5969,11 @@
       <c r="F10" s="1" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -5689,8 +5992,11 @@
       <c r="F11" s="7" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -5709,8 +6015,11 @@
       <c r="F12" s="4" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -5729,8 +6038,11 @@
       <c r="F13" s="7" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -5749,8 +6061,11 @@
       <c r="F14" s="4" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -5769,8 +6084,11 @@
       <c r="F15" s="7" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -5789,8 +6107,11 @@
       <c r="F16" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -5809,8 +6130,11 @@
       <c r="F17" s="7" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -5829,8 +6153,11 @@
       <c r="F18" s="4" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -5849,8 +6176,11 @@
       <c r="F19" s="7" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -5869,8 +6199,11 @@
       <c r="F20" s="4" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -5888,6 +6221,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>158</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1066</v>
       </c>
     </row>
   </sheetData>
@@ -5898,7 +6234,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E94D705-8DE7-4145-AD1D-2FF5088D0F88}">
   <sheetPr codeName="Sheet24"/>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -5906,9 +6242,10 @@
     <col min="3" max="3" width="59.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="78.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="53" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -5924,8 +6261,14 @@
       <c r="E1" s="10" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -5941,8 +6284,14 @@
       <c r="E2" s="4" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -5958,8 +6307,14 @@
       <c r="E3" s="7" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -5975,8 +6330,14 @@
       <c r="E4" s="7" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -5992,8 +6353,14 @@
       <c r="E5" s="4" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -6009,8 +6376,14 @@
       <c r="E6" s="7" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -6026,8 +6399,14 @@
       <c r="E7" s="4" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -6043,8 +6422,14 @@
       <c r="E8" s="7" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -6060,8 +6445,14 @@
       <c r="E9" s="4" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -6077,8 +6468,14 @@
       <c r="E10" s="1" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -6094,8 +6491,14 @@
       <c r="E11" s="7" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -6111,8 +6514,14 @@
       <c r="E12" s="4" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -6128,8 +6537,14 @@
       <c r="E13" s="7" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -6145,8 +6560,14 @@
       <c r="E14" s="4" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -6162,8 +6583,14 @@
       <c r="E15" s="7" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -6179,8 +6606,14 @@
       <c r="E16" s="4" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -6196,8 +6629,14 @@
       <c r="E17" s="7" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -6213,8 +6652,14 @@
       <c r="E18" s="4" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -6230,8 +6675,14 @@
       <c r="E19" s="7" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -6247,8 +6698,14 @@
       <c r="E20" s="4" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -6263,6 +6720,12 @@
       </c>
       <c r="E21" s="4" t="s">
         <v>234</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1065</v>
       </c>
     </row>
   </sheetData>
@@ -6273,7 +6736,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D03BF4A-1A9E-473D-9AB6-8164A430FD21}">
   <sheetPr codeName="Sheet23"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -6284,7 +6747,7 @@
     <col min="6" max="6" width="44.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -6303,8 +6766,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -6323,8 +6789,11 @@
       <c r="F2" s="4" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -6343,8 +6812,11 @@
       <c r="F3" s="7" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -6363,8 +6835,11 @@
       <c r="F4" s="7" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -6383,8 +6858,11 @@
       <c r="F5" s="4" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -6403,8 +6881,11 @@
       <c r="F6" s="7" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -6423,8 +6904,11 @@
       <c r="F7" s="4" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -6443,8 +6927,11 @@
       <c r="F8" s="7" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -6463,8 +6950,11 @@
       <c r="F9" s="4" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -6483,8 +6973,11 @@
       <c r="F10" s="1" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -6503,8 +6996,11 @@
       <c r="F11" s="7" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -6523,8 +7019,11 @@
       <c r="F12" s="4" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -6543,8 +7042,11 @@
       <c r="F13" s="7" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -6563,8 +7065,11 @@
       <c r="F14" s="4" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -6583,8 +7088,11 @@
       <c r="F15" s="7" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -6603,8 +7111,11 @@
       <c r="F16" s="4" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -6623,8 +7134,11 @@
       <c r="F17" s="7" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -6643,8 +7157,11 @@
       <c r="F18" s="4" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -6663,8 +7180,11 @@
       <c r="F19" s="7" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -6683,8 +7203,11 @@
       <c r="F20" s="4" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -6702,6 +7225,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>311</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1066</v>
       </c>
     </row>
   </sheetData>
@@ -6712,7 +7238,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EDFEBF7-4179-46E5-B518-2E67C214BE6B}">
   <sheetPr codeName="Sheet22"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -6723,7 +7249,7 @@
     <col min="6" max="6" width="48.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -6742,8 +7268,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -6762,8 +7291,11 @@
       <c r="F2" s="4" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -6782,8 +7314,11 @@
       <c r="F3" s="7" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -6802,8 +7337,11 @@
       <c r="F4" s="7" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -6822,8 +7360,11 @@
       <c r="F5" s="4" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -6842,8 +7383,11 @@
       <c r="F6" s="7" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -6862,8 +7406,11 @@
       <c r="F7" s="4" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -6882,8 +7429,11 @@
       <c r="F8" s="7" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -6902,8 +7452,11 @@
       <c r="F9" s="4" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -6922,8 +7475,11 @@
       <c r="F10" s="1" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -6942,8 +7498,11 @@
       <c r="F11" s="7" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -6962,8 +7521,11 @@
       <c r="F12" s="4" t="s">
         <v>444</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -6982,8 +7544,11 @@
       <c r="F13" s="7" t="s">
         <v>440</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -7002,8 +7567,11 @@
       <c r="F14" s="4" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -7022,8 +7590,11 @@
       <c r="F15" s="7" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -7042,8 +7613,11 @@
       <c r="F16" s="4" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -7062,8 +7636,11 @@
       <c r="F17" s="7" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -7082,8 +7659,11 @@
       <c r="F18" s="4" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -7102,8 +7682,11 @@
       <c r="F19" s="7" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -7122,8 +7705,11 @@
       <c r="F20" s="4" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -7141,6 +7727,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>401</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1066</v>
       </c>
     </row>
   </sheetData>
@@ -7151,7 +7740,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10EC635B-296D-4097-BDB4-A1AE6EF24EDD}">
   <sheetPr codeName="Sheet21"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -7162,7 +7751,7 @@
     <col min="6" max="6" width="51.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -7181,8 +7770,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -7201,8 +7793,11 @@
       <c r="F2" s="4" t="s">
         <v>547</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -7221,8 +7816,11 @@
       <c r="F3" s="7" t="s">
         <v>496</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -7241,8 +7839,11 @@
       <c r="F4" s="7" t="s">
         <v>486</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -7261,8 +7862,11 @@
       <c r="F5" s="4" t="s">
         <v>481</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -7281,8 +7885,11 @@
       <c r="F6" s="7" t="s">
         <v>476</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -7301,8 +7908,11 @@
       <c r="F7" s="4" t="s">
         <v>471</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -7321,8 +7931,11 @@
       <c r="F8" s="7" t="s">
         <v>466</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -7341,8 +7954,11 @@
       <c r="F9" s="4" t="s">
         <v>461</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -7361,8 +7977,11 @@
       <c r="F10" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -7381,8 +8000,11 @@
       <c r="F11" s="7" t="s">
         <v>542</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -7401,8 +8023,11 @@
       <c r="F12" s="4" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -7421,8 +8046,11 @@
       <c r="F13" s="7" t="s">
         <v>534</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -7441,8 +8069,11 @@
       <c r="F14" s="4" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -7461,8 +8092,11 @@
       <c r="F15" s="7" t="s">
         <v>524</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -7481,8 +8115,11 @@
       <c r="F16" s="4" t="s">
         <v>519</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -7501,8 +8138,11 @@
       <c r="F17" s="7" t="s">
         <v>514</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -7521,8 +8161,11 @@
       <c r="F18" s="4" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -7541,8 +8184,11 @@
       <c r="F19" s="7" t="s">
         <v>506</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -7561,8 +8207,11 @@
       <c r="F20" s="4" t="s">
         <v>501</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -7580,6 +8229,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>491</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1067</v>
       </c>
     </row>
   </sheetData>
@@ -7590,7 +8242,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52A71D50-AB40-4CBC-8665-B7236F91316D}">
   <sheetPr codeName="Sheet20"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -7601,7 +8253,7 @@
     <col min="6" max="6" width="36" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -7620,8 +8272,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -7640,8 +8295,11 @@
       <c r="F2" s="4" t="s">
         <v>620</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -7660,8 +8318,11 @@
       <c r="F3" s="7" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -7680,8 +8341,11 @@
       <c r="F4" s="7" t="s">
         <v>578</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -7700,8 +8364,11 @@
       <c r="F5" s="4" t="s">
         <v>573</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -7720,8 +8387,11 @@
       <c r="F6" s="7" t="s">
         <v>568</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -7740,8 +8410,11 @@
       <c r="F7" s="4" t="s">
         <v>563</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -7760,8 +8433,11 @@
       <c r="F8" s="7" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -7780,8 +8456,11 @@
       <c r="F9" s="4" t="s">
         <v>553</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -7800,8 +8479,11 @@
       <c r="F10" s="1" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -7820,8 +8502,11 @@
       <c r="F11" s="7" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -7840,8 +8525,11 @@
       <c r="F12" s="4" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -7860,8 +8548,11 @@
       <c r="F13" s="7" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -7880,8 +8571,11 @@
       <c r="F14" s="4" t="s">
         <v>607</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -7900,8 +8594,11 @@
       <c r="F15" s="7" t="s">
         <v>603</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -7920,8 +8617,11 @@
       <c r="F16" s="4" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -7940,8 +8640,11 @@
       <c r="F17" s="7" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -7960,8 +8663,11 @@
       <c r="F18" s="4" t="s">
         <v>592</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -7980,8 +8686,11 @@
       <c r="F19" s="7" t="s">
         <v>591</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -8000,8 +8709,11 @@
       <c r="F20" s="4" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -8019,6 +8731,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>583</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1064</v>
       </c>
     </row>
   </sheetData>
@@ -8029,7 +8744,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBA26D0B-1CD2-460D-B2DA-F9A6F5BEEEA8}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -8040,7 +8755,7 @@
     <col min="6" max="6" width="57.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -8059,8 +8774,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -8079,8 +8797,11 @@
       <c r="F2" s="4" t="s">
         <v>717</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -8099,8 +8820,11 @@
       <c r="F3" s="7" t="s">
         <v>662</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -8119,8 +8843,11 @@
       <c r="F4" s="7" t="s">
         <v>652</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -8139,8 +8866,11 @@
       <c r="F5" s="4" t="s">
         <v>647</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -8159,8 +8889,11 @@
       <c r="F6" s="7" t="s">
         <v>642</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -8179,8 +8912,11 @@
       <c r="F7" s="4" t="s">
         <v>637</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -8199,8 +8935,11 @@
       <c r="F8" s="7" t="s">
         <v>632</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -8219,8 +8958,11 @@
       <c r="F9" s="4" t="s">
         <v>627</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -8239,8 +8981,11 @@
       <c r="F10" s="1" t="s">
         <v>622</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -8259,8 +9004,11 @@
       <c r="F11" s="7" t="s">
         <v>712</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -8279,8 +9027,11 @@
       <c r="F12" s="4" t="s">
         <v>707</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -8299,8 +9050,11 @@
       <c r="F13" s="7" t="s">
         <v>702</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -8319,8 +9073,11 @@
       <c r="F14" s="4" t="s">
         <v>697</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -8339,8 +9096,11 @@
       <c r="F15" s="7" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -8359,8 +9119,11 @@
       <c r="F16" s="4" t="s">
         <v>687</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -8379,8 +9142,11 @@
       <c r="F17" s="7" t="s">
         <v>682</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -8399,8 +9165,11 @@
       <c r="F18" s="4" t="s">
         <v>677</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -8419,8 +9188,11 @@
       <c r="F19" s="7" t="s">
         <v>672</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -8439,8 +9211,11 @@
       <c r="F20" s="4" t="s">
         <v>667</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -8458,6 +9233,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>657</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1065</v>
       </c>
     </row>
   </sheetData>
@@ -8468,7 +9246,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84BB32D4-2C65-413B-AA5F-A44F4E79B9E5}">
   <sheetPr codeName="Sheet18"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -8476,7 +9254,7 @@
     <col min="6" max="6" width="64" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -8495,8 +9273,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -8515,8 +9296,11 @@
       <c r="F2" s="4" t="s">
         <v>796</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>53</v>
       </c>
@@ -8535,8 +9319,11 @@
       <c r="F3" s="7" t="s">
         <v>761</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>41</v>
       </c>
@@ -8555,8 +9342,11 @@
       <c r="F4" s="7" t="s">
         <v>751</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
@@ -8575,8 +9365,11 @@
       <c r="F5" s="4" t="s">
         <v>746</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -8595,8 +9388,11 @@
       <c r="F6" s="7" t="s">
         <v>742</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -8615,8 +9411,11 @@
       <c r="F7" s="4" t="s">
         <v>737</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -8635,8 +9434,11 @@
       <c r="F8" s="7" t="s">
         <v>732</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -8655,8 +9457,11 @@
       <c r="F9" s="4" t="s">
         <v>727</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -8675,8 +9480,11 @@
       <c r="F10" s="1" t="s">
         <v>722</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -8695,8 +9503,11 @@
       <c r="F11" s="7" t="s">
         <v>793</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -8715,8 +9526,11 @@
       <c r="F12" s="4" t="s">
         <v>759</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -8735,8 +9549,11 @@
       <c r="F13" s="7" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -8755,8 +9572,11 @@
       <c r="F14" s="4" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -8775,8 +9595,11 @@
       <c r="F15" s="7" t="s">
         <v>725</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -8795,8 +9618,11 @@
       <c r="F16" s="4" t="s">
         <v>780</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -8815,8 +9641,11 @@
       <c r="F17" s="7" t="s">
         <v>778</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>71</v>
       </c>
@@ -8835,8 +9664,11 @@
       <c r="F18" s="4" t="s">
         <v>727</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
@@ -8855,8 +9687,11 @@
       <c r="F19" s="7" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>59</v>
       </c>
@@ -8875,8 +9710,11 @@
       <c r="F20" s="4" t="s">
         <v>766</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>47</v>
       </c>
@@ -8894,6 +9732,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>756</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1067</v>
       </c>
     </row>
   </sheetData>

</xml_diff>